<commit_message>
ISO W10 sapuan xlsx OPS dan ISMS (14 dokumen)
Tiap dokumen lolos gerbang mesin W10 (reports/w10/gates/KEY.json) dan
pemeriksa bahasa buta (qa/KEY.w10.json, semua skor >= 4). OPS-FRM-04, 08, 09
dan ISMS-REG-02 lolos di putaran 2 setelah perbaikan op format cetak.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BhkCQM7h3krZb9kjY2Nate
</commit_message>
<xml_diff>
--- a/out/07_Ops/SNX-OPS-FRM-01 Project Plan Scope Timeline (Rev00 DRAFT).xlsx
+++ b/out/07_Ops/SNX-OPS-FRM-01 Project Plan Scope Timeline (Rev00 DRAFT).xlsx
@@ -17,10 +17,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholder" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Daftar'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Checklist G1'!$A$4:$F$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Checklist G1'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'WBS dan Timeline'!$A$4:$M$104</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'WBS dan Timeline'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Milestone'!$A$4:$G$24</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Milestone'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Stakeholder'!$A$4:$G$20</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Stakeholder'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -174,7 +179,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -340,6 +345,30 @@
     </xf>
     <xf numFmtId="9" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -749,8 +778,15 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="30">
-      <c r="A4" s="33" t="inlineStr">
+    <row r="3" s="30">
+      <c r="A3" s="56" t="n"/>
+      <c r="B3" s="56" t="n"/>
+      <c r="C3" s="56" t="n"/>
+      <c r="D3" s="56" t="n"/>
+      <c r="E3" s="56" t="n"/>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" s="30">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>Nomor dokumen</t>
         </is>
@@ -760,9 +796,12 @@
           <t>SNX-OPS-FRM-01</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="30">
-      <c r="A5" s="33" t="inlineStr">
+      <c r="C4" s="56" t="n"/>
+      <c r="D4" s="56" t="n"/>
+      <c r="E4" s="56" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="30">
+      <c r="A5" s="50" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
@@ -772,9 +811,12 @@
           <t>Project Plan, Scope &amp; Timeline Records</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="30">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="C5" s="56" t="n"/>
+      <c r="D5" s="56" t="n"/>
+      <c r="E5" s="56" t="n"/>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="30">
+      <c r="A6" s="50" t="inlineStr">
         <is>
           <t>Revisi</t>
         </is>
@@ -784,9 +826,12 @@
           <t>00 (DRAFT)</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="30">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="C6" s="56" t="n"/>
+      <c r="D6" s="56" t="n"/>
+      <c r="E6" s="56" t="n"/>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="30">
+      <c r="A7" s="50" t="inlineStr">
         <is>
           <t>Tanggal draft</t>
         </is>
@@ -796,9 +841,12 @@
           <t>13 Oktober 2026</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="30">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="C7" s="56" t="n"/>
+      <c r="D7" s="56" t="n"/>
+      <c r="E7" s="56" t="n"/>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="30">
+      <c r="A8" s="50" t="inlineStr">
         <is>
           <t>Tanggal efektif</t>
         </is>
@@ -808,9 +856,12 @@
           <t>Ditetapkan saat pengesahan</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="30">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="C8" s="56" t="n"/>
+      <c r="D8" s="56" t="n"/>
+      <c r="E8" s="56" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="30">
+      <c r="A9" s="50" t="inlineStr">
         <is>
           <t>Klasifikasi</t>
         </is>
@@ -820,9 +871,12 @@
           <t>RESTRICTED (Internal)</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="30">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="C9" s="56" t="n"/>
+      <c r="D9" s="56" t="n"/>
+      <c r="E9" s="56" t="n"/>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="30">
+      <c r="A10" s="50" t="inlineStr">
         <is>
           <t>Pemilik dokumen</t>
         </is>
@@ -832,9 +886,12 @@
           <t>Project Manager</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="30">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="C10" s="56" t="n"/>
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="56" t="n"/>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="30">
+      <c r="A11" s="50" t="inlineStr">
         <is>
           <t>Disetujui oleh</t>
         </is>
@@ -844,9 +901,12 @@
           <t>Samuel Kristanto Utomo / President Director</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="30">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="C11" s="56" t="n"/>
+      <c r="D11" s="56" t="n"/>
+      <c r="E11" s="56" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="30">
+      <c r="A12" s="50" t="inlineStr">
         <is>
           <t>Acuan ISO 9001:2015</t>
         </is>
@@ -856,9 +916,12 @@
           <t>Klausul 8.1, 8.2.2</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="30">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="C12" s="56" t="n"/>
+      <c r="D12" s="56" t="n"/>
+      <c r="E12" s="56" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="30">
+      <c r="A13" s="50" t="inlineStr">
         <is>
           <t>Acuan ISO/IEC 27001:2022</t>
         </is>
@@ -868,9 +931,12 @@
           <t>Kontrol Annex A 5.8</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="30">
-      <c r="A14" s="33" t="inlineStr">
+      <c r="C13" s="56" t="n"/>
+      <c r="D13" s="56" t="n"/>
+      <c r="E13" s="56" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1" s="30">
+      <c r="A14" s="50" t="inlineStr">
         <is>
           <t>Masa simpan record</t>
         </is>
@@ -880,141 +946,203 @@
           <t>Durasi kontrak + 3 tahun</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="23.85" customHeight="1" s="30">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="C14" s="56" t="n"/>
+      <c r="D14" s="56" t="n"/>
+      <c r="E14" s="56" t="n"/>
+    </row>
+    <row r="15" ht="43.5" customHeight="1" s="30">
+      <c r="A15" s="50" t="inlineStr">
         <is>
           <t>Tujuan</t>
         </is>
       </c>
       <c r="B15" s="34" t="inlineStr">
         <is>
-          <t>Merekam rencana proyek: checklist penerimaan G1, project charter, WBS dan jadwal, milestone, serta stakeholder dan komunikasi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="30">
-      <c r="A17" s="35" t="inlineStr">
+          <t>Mencatat rencana proyek: checklist penerimaan G1, project charter, WBS dan jadwal, milestone, serta stakeholder dan rencana komunikasi.</t>
+        </is>
+      </c>
+      <c r="C15" s="56" t="n"/>
+      <c r="D15" s="56" t="n"/>
+      <c r="E15" s="56" t="n"/>
+    </row>
+    <row r="16" s="30">
+      <c r="A16" s="56" t="n"/>
+      <c r="B16" s="56" t="n"/>
+      <c r="C16" s="56" t="n"/>
+      <c r="D16" s="56" t="n"/>
+      <c r="E16" s="56" t="n"/>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="30">
+      <c r="A17" s="57" t="inlineStr">
         <is>
           <t>Cara pakai</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="30">
-      <c r="A18" s="36" t="inlineStr">
+      <c r="B17" s="56" t="n"/>
+      <c r="C17" s="56" t="n"/>
+      <c r="D17" s="56" t="n"/>
+      <c r="E17" s="56" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="30">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
       <c r="B18" s="37" t="inlineStr">
         <is>
-          <t>Salin file ini per proyek; ganti nama menjadi FRM-01_&lt;KodeProyek&gt;.xlsx.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="30">
-      <c r="A19" s="36" t="inlineStr">
+          <t>Gunakan satu file untuk satu proyek, dengan nama FRM-01_&lt;KodeProyek&gt;.xlsx.</t>
+        </is>
+      </c>
+      <c r="C18" s="56" t="n"/>
+      <c r="D18" s="56" t="n"/>
+      <c r="E18" s="56" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1" s="30">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Isi Checklist G1 sebelum proyek dimulai; proyek tidak dimulai bila ada butir Belum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="23.85" customHeight="1" s="30">
-      <c r="A20" s="36" t="inlineStr">
+          <t>Isi Checklist G1 sebelum proyek dimulai. Proyek belum boleh dimulai jika masih ada butir berstatus Belum.</t>
+        </is>
+      </c>
+      <c r="C19" s="56" t="n"/>
+      <c r="D19" s="56" t="n"/>
+      <c r="E19" s="56" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1" s="30">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Isi Project Charter, lalu WBS dan Timeline. Durasi dan progres keseluruhan dihitung otomatis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="23.85" customHeight="1" s="30">
-      <c r="A21" s="36" t="inlineStr">
+          <t>Isi Project Charter, lalu sheet WBS dan Timeline. Durasi dan progres keseluruhan terisi otomatis.</t>
+        </is>
+      </c>
+      <c r="C20" s="56" t="n"/>
+      <c r="D20" s="56" t="n"/>
+      <c r="E20" s="56" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1" s="30">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
       <c r="B21" s="37" t="inlineStr">
         <is>
-          <t>Perbarui kolom Progres dan Status minimal mingguan (SNX-OPS-SOP-01 Bagian 6.4).</t>
-        </is>
-      </c>
+          <t>Perbarui kolom Progres dan Status paling sedikit sekali seminggu, sesuai SNX-OPS-SOP-01 butir 6.4.</t>
+        </is>
+      </c>
+      <c r="C21" s="56" t="n"/>
+      <c r="D21" s="56" t="n"/>
+      <c r="E21" s="56" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="30">
-      <c r="A22" s="36" t="n"/>
+      <c r="A22" s="37" t="n"/>
       <c r="B22" s="37" t="n"/>
-    </row>
-    <row r="23"/>
-    <row r="24" ht="15" customHeight="1" s="30">
-      <c r="A24" s="35" t="inlineStr">
+      <c r="C22" s="56" t="n"/>
+      <c r="D22" s="56" t="n"/>
+      <c r="E22" s="56" t="n"/>
+    </row>
+    <row r="23" s="30">
+      <c r="A23" s="56" t="n"/>
+      <c r="B23" s="56" t="n"/>
+      <c r="C23" s="56" t="n"/>
+      <c r="D23" s="56" t="n"/>
+      <c r="E23" s="56" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="30">
+      <c r="A24" s="57" t="inlineStr">
         <is>
           <t>Legenda warna</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="30">
-      <c r="A25" s="38" t="n"/>
-      <c r="B25" s="36" t="inlineStr">
+      <c r="B24" s="56" t="n"/>
+      <c r="C24" s="56" t="n"/>
+      <c r="D24" s="56" t="n"/>
+      <c r="E24" s="56" t="n"/>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="30">
+      <c r="A25" s="51" t="n"/>
+      <c r="B25" s="37" t="inlineStr">
         <is>
           <t>Sel input: diisi pengguna</t>
         </is>
       </c>
+      <c r="C25" s="56" t="n"/>
+      <c r="D25" s="56" t="n"/>
+      <c r="E25" s="56" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="30">
-      <c r="A26" s="39" t="n"/>
-      <c r="B26" s="36" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="30">
-      <c r="A27" s="40" t="n"/>
-      <c r="B27" s="36" t="inlineStr">
+      <c r="A26" s="58" t="n"/>
+      <c r="B26" s="37" t="n"/>
+      <c r="C26" s="56" t="n"/>
+      <c r="D26" s="56" t="n"/>
+      <c r="E26" s="56" t="n"/>
+    </row>
+    <row r="27" ht="16.5" customHeight="1" s="30">
+      <c r="A27" s="59" t="n"/>
+      <c r="B27" s="37" t="inlineStr">
         <is>
           <t>Sel rumus: jangan diubah</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="30">
-      <c r="A29" s="35" t="inlineStr">
+      <c r="C27" s="56" t="n"/>
+      <c r="D27" s="56" t="n"/>
+      <c r="E27" s="56" t="n"/>
+    </row>
+    <row r="28" s="30">
+      <c r="A28" s="56" t="n"/>
+      <c r="B28" s="56" t="n"/>
+      <c r="C28" s="56" t="n"/>
+      <c r="D28" s="56" t="n"/>
+      <c r="E28" s="56" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="30">
+      <c r="A29" s="57" t="inlineStr">
         <is>
           <t>Riwayat revisi</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="30">
-      <c r="A30" s="41" t="inlineStr">
+      <c r="B29" s="56" t="n"/>
+      <c r="C29" s="56" t="n"/>
+      <c r="D29" s="56" t="n"/>
+      <c r="E29" s="56" t="n"/>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="30">
+      <c r="A30" s="45" t="inlineStr">
         <is>
           <t>Revisi</t>
         </is>
       </c>
-      <c r="B30" s="41" t="inlineStr">
+      <c r="B30" s="45" t="inlineStr">
         <is>
           <t>Tanggal</t>
         </is>
       </c>
-      <c r="C30" s="41" t="inlineStr">
+      <c r="C30" s="45" t="inlineStr">
         <is>
           <t>Uraian perubahan</t>
         </is>
       </c>
-      <c r="D30" s="41" t="inlineStr">
+      <c r="D30" s="45" t="inlineStr">
         <is>
           <t>Disusun</t>
         </is>
       </c>
-      <c r="E30" s="41" t="inlineStr">
+      <c r="E30" s="45" t="inlineStr">
         <is>
           <t>Disetujui</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="23.85" customHeight="1" s="30">
+    <row r="31" ht="30" customHeight="1" s="30">
       <c r="A31" s="34" t="inlineStr">
         <is>
           <t>00</t>
@@ -1048,77 +1176,91 @@
       <c r="D32" s="34" t="n"/>
       <c r="E32" s="34" t="n"/>
     </row>
-    <row r="33"/>
-    <row r="34" ht="15" customHeight="1" s="30">
-      <c r="A34" s="35" t="inlineStr">
+    <row r="33" s="30">
+      <c r="A33" s="56" t="n"/>
+      <c r="B33" s="56" t="n"/>
+      <c r="C33" s="56" t="n"/>
+      <c r="D33" s="56" t="n"/>
+      <c r="E33" s="56" t="n"/>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="30">
+      <c r="A34" s="57" t="inlineStr">
         <is>
           <t>Pengesahan</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="30">
-      <c r="A35" s="41" t="inlineStr">
+      <c r="B34" s="56" t="n"/>
+      <c r="C34" s="56" t="n"/>
+      <c r="D34" s="56" t="n"/>
+      <c r="E34" s="56" t="n"/>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="30">
+      <c r="A35" s="45" t="inlineStr">
         <is>
           <t>Peran</t>
         </is>
       </c>
-      <c r="B35" s="41" t="inlineStr">
+      <c r="B35" s="45" t="inlineStr">
         <is>
           <t>Nama dan jabatan</t>
         </is>
       </c>
-      <c r="C35" s="41" t="inlineStr">
+      <c r="C35" s="45" t="inlineStr">
         <is>
           <t>Tanda tangan</t>
         </is>
       </c>
-      <c r="D35" s="41" t="inlineStr">
+      <c r="D35" s="45" t="inlineStr">
         <is>
           <t>Tanggal</t>
         </is>
       </c>
+      <c r="E35" s="56" t="n"/>
     </row>
     <row r="36" ht="27.75" customHeight="1" s="30">
-      <c r="A36" s="42" t="inlineStr">
+      <c r="A36" s="34" t="inlineStr">
         <is>
           <t>Disusun oleh</t>
         </is>
       </c>
-      <c r="B36" s="42" t="inlineStr">
+      <c r="B36" s="34" t="inlineStr">
         <is>
           <t>Erik Dwi Yanto / Technical/Operation Engineer L1</t>
         </is>
       </c>
-      <c r="C36" s="42" t="n"/>
-      <c r="D36" s="42" t="n"/>
+      <c r="C36" s="34" t="n"/>
+      <c r="D36" s="34" t="n"/>
+      <c r="E36" s="56" t="n"/>
     </row>
     <row r="37" ht="27.75" customHeight="1" s="30">
-      <c r="A37" s="42" t="inlineStr">
+      <c r="A37" s="34" t="inlineStr">
         <is>
           <t>Diperiksa oleh</t>
         </is>
       </c>
-      <c r="B37" s="42" t="inlineStr">
+      <c r="B37" s="34" t="inlineStr">
         <is>
           <t>Fani Fatullah / VP Tech Operation and Services</t>
         </is>
       </c>
-      <c r="C37" s="42" t="n"/>
-      <c r="D37" s="42" t="n"/>
+      <c r="C37" s="34" t="n"/>
+      <c r="D37" s="34" t="n"/>
+      <c r="E37" s="56" t="n"/>
     </row>
     <row r="38" ht="27.75" customHeight="1" s="30">
-      <c r="A38" s="42" t="inlineStr">
+      <c r="A38" s="34" t="inlineStr">
         <is>
           <t>Disetujui oleh</t>
         </is>
       </c>
-      <c r="B38" s="42" t="inlineStr">
+      <c r="B38" s="34" t="inlineStr">
         <is>
           <t>Samuel Kristanto Utomo / President Director</t>
         </is>
       </c>
-      <c r="C38" s="42" t="n"/>
-      <c r="D38" s="42" t="n"/>
+      <c r="C38" s="34" t="n"/>
+      <c r="D38" s="34" t="n"/>
+      <c r="E38" s="56" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1162,106 +1304,110 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="29" min="1" max="2"/>
+    <col width="13" customWidth="1" style="30" min="2" max="2"/>
     <col width="18" customWidth="1" style="29" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="30">
-      <c r="A1" s="44" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="30">
+      <c r="A1" s="60" t="inlineStr">
         <is>
           <t>Status tugas</t>
         </is>
       </c>
-      <c r="B1" s="44" t="inlineStr">
+      <c r="B1" s="60" t="inlineStr">
         <is>
           <t>Status G1</t>
         </is>
       </c>
-      <c r="C1" s="44" t="inlineStr">
+      <c r="C1" s="60" t="inlineStr">
         <is>
           <t>Status milestone</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="30">
-      <c r="A2" s="36" t="inlineStr">
+    <row r="2" ht="16.5" customHeight="1" s="30">
+      <c r="A2" s="61" t="inlineStr">
         <is>
           <t>Belum mulai</t>
         </is>
       </c>
-      <c r="B2" s="36" t="inlineStr">
+      <c r="B2" s="61" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
-      <c r="C2" s="36" t="inlineStr">
+      <c r="C2" s="61" t="inlineStr">
         <is>
           <t>Sesuai rencana</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="30">
-      <c r="A3" s="36" t="inlineStr">
+    <row r="3" ht="16.5" customHeight="1" s="30">
+      <c r="A3" s="61" t="inlineStr">
         <is>
           <t>Berjalan</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
+      <c r="B3" s="61" t="inlineStr">
         <is>
           <t>Lolos</t>
         </is>
       </c>
-      <c r="C3" s="36" t="inlineStr">
+      <c r="C3" s="61" t="inlineStr">
         <is>
           <t>Berisiko</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="30">
-      <c r="A4" s="36" t="inlineStr">
+    <row r="4" ht="30" customHeight="1" s="30">
+      <c r="A4" s="61" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t>Tidak berlaku</t>
         </is>
       </c>
-      <c r="C4" s="36" t="inlineStr">
+      <c r="C4" s="61" t="inlineStr">
         <is>
           <t>Terlambat</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="30">
-      <c r="A5" s="36" t="inlineStr">
+    <row r="5" ht="16.5" customHeight="1" s="30">
+      <c r="A5" s="61" t="inlineStr">
         <is>
           <t>Tertunda</t>
         </is>
       </c>
-      <c r="C5" s="36" t="inlineStr">
+      <c r="B5" s="62" t="n"/>
+      <c r="C5" s="61" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="30">
-      <c r="A6" s="36" t="inlineStr">
+    <row r="6" ht="16.5" customHeight="1" s="30">
+      <c r="A6" s="61" t="inlineStr">
         <is>
           <t>Dibatalkan</t>
         </is>
       </c>
+      <c r="B6" s="62" t="n"/>
+      <c r="C6" s="62" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -1292,7 +1438,7 @@
     <row r="2" ht="15" customHeight="1" s="30">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>Pemilik gate: Service Delivery Manager. Gate LOLOS bila tidak ada butir berstatus Belum.</t>
+          <t>Pemilik gate: Service Delivery Manager. Gate LOLOS jika tidak ada butir berstatus Belum.</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1474,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="30">
+    <row r="5" ht="16.5" customHeight="1" s="30">
       <c r="A5" s="46" t="n">
         <v>1</v>
       </c>
@@ -1346,7 +1492,7 @@
       <c r="E5" s="47" t="n"/>
       <c r="F5" s="48" t="n"/>
     </row>
-    <row r="6" ht="15" customHeight="1" s="30">
+    <row r="6" ht="16.5" customHeight="1" s="30">
       <c r="A6" s="46" t="n">
         <v>2</v>
       </c>
@@ -1364,7 +1510,7 @@
       <c r="E6" s="47" t="n"/>
       <c r="F6" s="48" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1" s="30">
+    <row r="7" ht="30" customHeight="1" s="30">
       <c r="A7" s="46" t="n">
         <v>3</v>
       </c>
@@ -1382,7 +1528,7 @@
       <c r="E7" s="47" t="n"/>
       <c r="F7" s="48" t="n"/>
     </row>
-    <row r="8" ht="15" customHeight="1" s="30">
+    <row r="8" ht="16.5" customHeight="1" s="30">
       <c r="A8" s="46" t="n">
         <v>4</v>
       </c>
@@ -1400,7 +1546,7 @@
       <c r="E8" s="47" t="n"/>
       <c r="F8" s="48" t="n"/>
     </row>
-    <row r="9" ht="15" customHeight="1" s="30">
+    <row r="9" ht="30" customHeight="1" s="30">
       <c r="A9" s="46" t="n">
         <v>5</v>
       </c>
@@ -1418,7 +1564,7 @@
       <c r="E9" s="47" t="n"/>
       <c r="F9" s="48" t="n"/>
     </row>
-    <row r="10" ht="15" customHeight="1" s="30">
+    <row r="10" ht="30" customHeight="1" s="30">
       <c r="A10" s="46" t="n">
         <v>6</v>
       </c>
@@ -1436,7 +1582,7 @@
       <c r="E10" s="47" t="n"/>
       <c r="F10" s="48" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1" s="30">
+    <row r="11" ht="30" customHeight="1" s="30">
       <c r="A11" s="46" t="n">
         <v>7</v>
       </c>
@@ -1454,7 +1600,7 @@
       <c r="E11" s="47" t="n"/>
       <c r="F11" s="48" t="n"/>
     </row>
-    <row r="12" ht="23.85" customHeight="1" s="30">
+    <row r="12" ht="30" customHeight="1" s="30">
       <c r="A12" s="46" t="n">
         <v>8</v>
       </c>
@@ -1472,16 +1618,28 @@
       <c r="E12" s="47" t="n"/>
       <c r="F12" s="48" t="n"/>
     </row>
-    <row r="14" ht="15" customHeight="1" s="30">
-      <c r="B14" s="49" t="inlineStr">
+    <row r="13" s="30">
+      <c r="A13" s="62" t="n"/>
+      <c r="B13" s="62" t="n"/>
+      <c r="C13" s="62" t="n"/>
+      <c r="D13" s="62" t="n"/>
+      <c r="E13" s="62" t="n"/>
+      <c r="F13" s="62" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="30">
+      <c r="A14" s="62" t="n"/>
+      <c r="B14" s="63" t="inlineStr">
         <is>
           <t>Keputusan G1</t>
         </is>
       </c>
-      <c r="C14" s="49">
+      <c r="C14" s="63">
         <f>IF(COUNTIF(C5:C12,"Belum")=0,"LOLOS","TAHAN")</f>
         <v/>
       </c>
+      <c r="D14" s="62" t="n"/>
+      <c r="E14" s="62" t="n"/>
+      <c r="F14" s="62" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:F12"/>
@@ -1514,7 +1672,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
@@ -1696,7 +1854,7 @@
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -1714,11 +1872,13 @@
     <col width="38" customWidth="1" style="29" min="3" max="3"/>
     <col width="20" customWidth="1" style="29" min="4" max="4"/>
     <col width="12" customWidth="1" style="29" min="5" max="6"/>
+    <col width="13" customWidth="1" style="30" min="6" max="6"/>
     <col width="10" customWidth="1" style="29" min="7" max="7"/>
     <col width="26" customWidth="1" style="29" min="8" max="8"/>
     <col width="9" customWidth="1" style="29" min="9" max="10"/>
+    <col width="13" customWidth="1" style="30" min="10" max="10"/>
     <col width="13" customWidth="1" style="29" min="11" max="11"/>
-    <col width="12" customWidth="1" style="29" min="12" max="12"/>
+    <col width="15" customWidth="1" style="29" min="12" max="12"/>
     <col width="22" customWidth="1" style="29" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -1732,7 +1892,7 @@
     <row r="2" ht="15" customHeight="1" s="30">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>Bobot dalam persen (total 100). Progres 0% sampai 100%. Kolom Durasi dihitung otomatis (hari kalender).</t>
+          <t>Bobot ditulis dalam persen dengan total 100. Progres diisi 0% sampai 100%. Kolom Durasi terisi otomatis dalam hari kalender.</t>
         </is>
       </c>
       <c r="I2" s="49" t="inlineStr">
@@ -3993,7 +4153,7 @@
     <row r="2" ht="15" customHeight="1" s="30">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>Kanal resmi: email dan grup WhatsApp proyek. Kredensial tidak pernah dikirim melalui kanal ini.</t>
+          <t>Kanal resmi adalah email dan grup WhatsApp proyek. Kredensial tidak boleh dikirim melalui kanal ini.</t>
         </is>
       </c>
     </row>

</xml_diff>